<commit_message>
feat: mapa de ubicación (geopandas + proyecto QGIS), grupo tectónico y fotos del equipo
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/tabla_variables.xlsx
+++ b/data/tabla_variables.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="601" uniqueCount="306">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="609" uniqueCount="310">
   <si>
     <t>Variable</t>
   </si>
@@ -100,6 +100,9 @@
     <t>Expedition</t>
   </si>
   <si>
+    <t>Tectonic Group</t>
+  </si>
+  <si>
     <t>Alteration Grade</t>
   </si>
   <si>
@@ -322,6 +325,9 @@
     <t>Expedición o campaña de muestreo</t>
   </si>
   <si>
+    <t>Ambiente tectónico agrupado en tres clases (o mixto)</t>
+  </si>
+  <si>
     <t>Grado de alteración: 0 fresca, 1 leve, 2 moderada, 3 extensa, 4 casi total, 5 total</t>
   </si>
   <si>
@@ -541,6 +547,9 @@
     <t>geocronología</t>
   </si>
   <si>
+    <t>derivada de Tectonic Setting</t>
+  </si>
+  <si>
     <t>derivada de Sample Alteration</t>
   </si>
   <si>
@@ -767,6 +776,9 @@
   </si>
   <si>
     <t>1312 categorías</t>
+  </si>
+  <si>
+    <t>4 categorías (p. ej. dorsal y corteza oceanica, intraplaca y rift, margen convergente…)</t>
   </si>
   <si>
     <t>{0, 1, 2, 3, 4, 5}</t>
@@ -1289,7 +1301,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I75"/>
+  <dimension ref="A1:I76"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:9">
@@ -1326,25 +1338,25 @@
         <v>9</v>
       </c>
       <c r="B2" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C2" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="D2" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="E2" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="F2" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="G2" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="H2" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="I2">
         <v>99.5</v>
@@ -1355,25 +1367,25 @@
         <v>10</v>
       </c>
       <c r="B3" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C3" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="D3" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="E3" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="F3" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="G3" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="H3" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="I3">
         <v>100</v>
@@ -1384,25 +1396,25 @@
         <v>11</v>
       </c>
       <c r="B4" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C4" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="D4" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="E4" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="F4" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="G4" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="H4" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="I4">
         <v>100</v>
@@ -1413,25 +1425,25 @@
         <v>12</v>
       </c>
       <c r="B5" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C5" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="D5" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="E5" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="F5" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="G5" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="H5" t="s">
-        <v>235</v>
+        <v>238</v>
       </c>
       <c r="I5">
         <v>100</v>
@@ -1442,25 +1454,25 @@
         <v>13</v>
       </c>
       <c r="B6" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C6" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="D6" t="s">
+        <v>161</v>
+      </c>
+      <c r="E6" t="s">
         <v>159</v>
       </c>
-      <c r="E6" t="s">
-        <v>157</v>
-      </c>
       <c r="F6" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="G6" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="H6" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="I6">
         <v>100</v>
@@ -1471,25 +1483,25 @@
         <v>14</v>
       </c>
       <c r="B7" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C7" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="D7" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="E7" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="F7" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="G7" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="H7" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="I7">
         <v>100</v>
@@ -1500,25 +1512,25 @@
         <v>15</v>
       </c>
       <c r="B8" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C8" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="D8" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="E8" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="F8" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="G8" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="H8" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
       <c r="I8">
         <v>100</v>
@@ -1529,25 +1541,25 @@
         <v>16</v>
       </c>
       <c r="B9" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C9" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="D9" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="E9" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="F9" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="G9" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
       <c r="H9" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
       <c r="I9">
         <v>100</v>
@@ -1558,25 +1570,25 @@
         <v>17</v>
       </c>
       <c r="B10" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C10" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="D10" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="E10" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="F10" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="G10" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
       <c r="H10" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="I10">
         <v>100</v>
@@ -1587,25 +1599,25 @@
         <v>18</v>
       </c>
       <c r="B11" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C11" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="D11" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="E11" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="F11" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="G11" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="H11" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
       <c r="I11">
         <v>99.8</v>
@@ -1616,25 +1628,25 @@
         <v>19</v>
       </c>
       <c r="B12" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C12" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="D12" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="E12" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="F12" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="G12" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="H12" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="I12">
         <v>99.8</v>
@@ -1645,25 +1657,25 @@
         <v>20</v>
       </c>
       <c r="B13" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C13" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="D13" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="E13" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="F13" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="G13" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="H13" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
       <c r="I13">
         <v>24.9</v>
@@ -1674,25 +1686,25 @@
         <v>21</v>
       </c>
       <c r="B14" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C14" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="D14" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="E14" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="F14" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="G14" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="H14" t="s">
-        <v>244</v>
+        <v>247</v>
       </c>
       <c r="I14">
         <v>22.1</v>
@@ -1703,25 +1715,25 @@
         <v>22</v>
       </c>
       <c r="B15" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C15" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="D15" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="E15" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="F15" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="G15" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
       <c r="H15" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
       <c r="I15">
         <v>53.5</v>
@@ -1732,25 +1744,25 @@
         <v>23</v>
       </c>
       <c r="B16" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C16" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="D16" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="E16" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="F16" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="G16" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
       <c r="H16" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="I16">
         <v>39.2</v>
@@ -1761,25 +1773,25 @@
         <v>24</v>
       </c>
       <c r="B17" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C17" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="D17" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="E17" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="F17" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="G17" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="H17" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
       <c r="I17">
         <v>10.5</v>
@@ -1790,25 +1802,25 @@
         <v>25</v>
       </c>
       <c r="B18" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C18" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="D18" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="E18" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="F18" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="G18" t="s">
-        <v>230</v>
+        <v>233</v>
       </c>
       <c r="H18" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="I18">
         <v>5.5</v>
@@ -1819,25 +1831,25 @@
         <v>26</v>
       </c>
       <c r="B19" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C19" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="D19" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="E19" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="F19" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="G19" t="s">
-        <v>230</v>
+        <v>233</v>
       </c>
       <c r="H19" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="I19">
         <v>7.9</v>
@@ -1848,25 +1860,25 @@
         <v>27</v>
       </c>
       <c r="B20" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C20" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="D20" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="E20" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="F20" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="G20" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="H20" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="I20">
         <v>99.90000000000001</v>
@@ -1877,28 +1889,28 @@
         <v>28</v>
       </c>
       <c r="B21" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C21" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="D21" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="E21" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="F21" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="G21" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="H21" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
       <c r="I21">
-        <v>20.8</v>
+        <v>99.8</v>
       </c>
     </row>
     <row r="22" spans="1:9">
@@ -1906,28 +1918,28 @@
         <v>29</v>
       </c>
       <c r="B22" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C22" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="D22" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="E22" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="F22" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="G22" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="H22" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="I22">
-        <v>35.7</v>
+        <v>20.8</v>
       </c>
     </row>
     <row r="23" spans="1:9">
@@ -1935,28 +1947,28 @@
         <v>30</v>
       </c>
       <c r="B23" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C23" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="D23" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="E23" t="s">
         <v>163</v>
       </c>
       <c r="F23" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="G23" t="s">
-        <v>231</v>
+        <v>158</v>
       </c>
       <c r="H23" t="s">
-        <v>253</v>
+        <v>256</v>
       </c>
       <c r="I23">
-        <v>100</v>
+        <v>35.7</v>
       </c>
     </row>
     <row r="24" spans="1:9">
@@ -1964,28 +1976,28 @@
         <v>31</v>
       </c>
       <c r="B24" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C24" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="D24" t="s">
         <v>160</v>
       </c>
       <c r="E24" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="F24" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="G24" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="H24" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
       <c r="I24">
-        <v>35.7</v>
+        <v>100</v>
       </c>
     </row>
     <row r="25" spans="1:9">
@@ -1993,28 +2005,28 @@
         <v>32</v>
       </c>
       <c r="B25" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C25" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="D25" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="E25" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="F25" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="G25" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
       <c r="H25" t="s">
-        <v>255</v>
+        <v>258</v>
       </c>
       <c r="I25">
-        <v>35.9</v>
+        <v>35.7</v>
       </c>
     </row>
     <row r="26" spans="1:9">
@@ -2022,28 +2034,28 @@
         <v>33</v>
       </c>
       <c r="B26" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C26" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="D26" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="E26" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="F26" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="G26" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
       <c r="H26" t="s">
-        <v>256</v>
+        <v>259</v>
       </c>
       <c r="I26">
-        <v>14.6</v>
+        <v>35.9</v>
       </c>
     </row>
     <row r="27" spans="1:9">
@@ -2051,28 +2063,28 @@
         <v>34</v>
       </c>
       <c r="B27" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C27" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="D27" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="E27" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="F27" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="G27" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
       <c r="H27" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
       <c r="I27">
-        <v>8.1</v>
+        <v>14.6</v>
       </c>
     </row>
     <row r="28" spans="1:9">
@@ -2080,28 +2092,28 @@
         <v>35</v>
       </c>
       <c r="B28" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C28" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="D28" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="E28" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="F28" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="G28" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
       <c r="H28" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
       <c r="I28">
-        <v>13.8</v>
+        <v>8.1</v>
       </c>
     </row>
     <row r="29" spans="1:9">
@@ -2109,28 +2121,28 @@
         <v>36</v>
       </c>
       <c r="B29" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C29" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="D29" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="E29" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="F29" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="G29" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
       <c r="H29" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="I29">
-        <v>9.1</v>
+        <v>13.8</v>
       </c>
     </row>
     <row r="30" spans="1:9">
@@ -2138,28 +2150,28 @@
         <v>37</v>
       </c>
       <c r="B30" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C30" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="D30" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="E30" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="F30" t="s">
-        <v>178</v>
+        <v>185</v>
       </c>
       <c r="G30" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
       <c r="H30" t="s">
-        <v>260</v>
+        <v>263</v>
       </c>
       <c r="I30">
-        <v>35.7</v>
+        <v>9.1</v>
       </c>
     </row>
     <row r="31" spans="1:9">
@@ -2167,28 +2179,28 @@
         <v>38</v>
       </c>
       <c r="B31" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C31" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="D31" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="E31" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="F31" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="G31" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
       <c r="H31" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="I31">
-        <v>34.5</v>
+        <v>35.7</v>
       </c>
     </row>
     <row r="32" spans="1:9">
@@ -2196,28 +2208,28 @@
         <v>39</v>
       </c>
       <c r="B32" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C32" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="D32" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="E32" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="F32" t="s">
-        <v>178</v>
+        <v>186</v>
       </c>
       <c r="G32" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
       <c r="H32" t="s">
-        <v>262</v>
+        <v>265</v>
       </c>
       <c r="I32">
-        <v>35.8</v>
+        <v>34.5</v>
       </c>
     </row>
     <row r="33" spans="1:9">
@@ -2225,28 +2237,28 @@
         <v>40</v>
       </c>
       <c r="B33" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C33" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="D33" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="E33" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="F33" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="G33" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
       <c r="H33" t="s">
-        <v>263</v>
+        <v>266</v>
       </c>
       <c r="I33">
-        <v>34.5</v>
+        <v>35.8</v>
       </c>
     </row>
     <row r="34" spans="1:9">
@@ -2254,28 +2266,28 @@
         <v>41</v>
       </c>
       <c r="B34" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C34" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="D34" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="E34" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="F34" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="G34" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
       <c r="H34" t="s">
-        <v>264</v>
+        <v>267</v>
       </c>
       <c r="I34">
-        <v>34</v>
+        <v>34.5</v>
       </c>
     </row>
     <row r="35" spans="1:9">
@@ -2283,28 +2295,28 @@
         <v>42</v>
       </c>
       <c r="B35" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C35" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="D35" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="E35" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="F35" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="G35" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
       <c r="H35" t="s">
-        <v>265</v>
+        <v>268</v>
       </c>
       <c r="I35">
-        <v>30.2</v>
+        <v>34</v>
       </c>
     </row>
     <row r="36" spans="1:9">
@@ -2312,28 +2324,28 @@
         <v>43</v>
       </c>
       <c r="B36" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="C36" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="D36" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="E36" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="F36" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="G36" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
       <c r="H36" t="s">
-        <v>266</v>
+        <v>269</v>
       </c>
       <c r="I36">
-        <v>6.9</v>
+        <v>30.2</v>
       </c>
     </row>
     <row r="37" spans="1:9">
@@ -2341,28 +2353,28 @@
         <v>44</v>
       </c>
       <c r="B37" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C37" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="D37" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="E37" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="F37" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="G37" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
       <c r="H37" t="s">
-        <v>267</v>
+        <v>270</v>
       </c>
       <c r="I37">
-        <v>7.8</v>
+        <v>6.9</v>
       </c>
     </row>
     <row r="38" spans="1:9">
@@ -2370,28 +2382,28 @@
         <v>45</v>
       </c>
       <c r="B38" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C38" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="D38" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="E38" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="F38" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="G38" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
       <c r="H38" t="s">
-        <v>268</v>
+        <v>271</v>
       </c>
       <c r="I38">
-        <v>15.6</v>
+        <v>7.8</v>
       </c>
     </row>
     <row r="39" spans="1:9">
@@ -2399,28 +2411,28 @@
         <v>46</v>
       </c>
       <c r="B39" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="C39" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="D39" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="E39" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="F39" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="G39" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
       <c r="H39" t="s">
-        <v>269</v>
+        <v>272</v>
       </c>
       <c r="I39">
-        <v>8.699999999999999</v>
+        <v>15.6</v>
       </c>
     </row>
     <row r="40" spans="1:9">
@@ -2428,28 +2440,28 @@
         <v>47</v>
       </c>
       <c r="B40" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C40" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="D40" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="E40" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="F40" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="G40" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
       <c r="H40" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
       <c r="I40">
-        <v>8</v>
+        <v>8.699999999999999</v>
       </c>
     </row>
     <row r="41" spans="1:9">
@@ -2457,28 +2469,28 @@
         <v>48</v>
       </c>
       <c r="B41" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C41" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="D41" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="E41" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="F41" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="G41" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="H41" t="s">
-        <v>271</v>
+        <v>274</v>
       </c>
       <c r="I41">
-        <v>27.6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="42" spans="1:9">
@@ -2486,28 +2498,28 @@
         <v>49</v>
       </c>
       <c r="B42" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C42" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="D42" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="E42" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="F42" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="G42" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="H42" t="s">
-        <v>272</v>
+        <v>275</v>
       </c>
       <c r="I42">
-        <v>31.1</v>
+        <v>27.6</v>
       </c>
     </row>
     <row r="43" spans="1:9">
@@ -2515,28 +2527,28 @@
         <v>50</v>
       </c>
       <c r="B43" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C43" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="D43" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="E43" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="F43" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="G43" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="H43" t="s">
-        <v>273</v>
+        <v>276</v>
       </c>
       <c r="I43">
-        <v>25.1</v>
+        <v>31.1</v>
       </c>
     </row>
     <row r="44" spans="1:9">
@@ -2544,28 +2556,28 @@
         <v>51</v>
       </c>
       <c r="B44" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C44" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="D44" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="E44" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="F44" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="G44" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="H44" t="s">
-        <v>274</v>
+        <v>277</v>
       </c>
       <c r="I44">
-        <v>11.2</v>
+        <v>25.1</v>
       </c>
     </row>
     <row r="45" spans="1:9">
@@ -2573,28 +2585,28 @@
         <v>52</v>
       </c>
       <c r="B45" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C45" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="D45" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="E45" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="F45" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="G45" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="H45" t="s">
-        <v>275</v>
+        <v>278</v>
       </c>
       <c r="I45">
-        <v>15.2</v>
+        <v>11.2</v>
       </c>
     </row>
     <row r="46" spans="1:9">
@@ -2602,28 +2614,28 @@
         <v>53</v>
       </c>
       <c r="B46" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C46" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="D46" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="E46" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="F46" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="G46" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="H46" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="I46">
-        <v>27.5</v>
+        <v>15.2</v>
       </c>
     </row>
     <row r="47" spans="1:9">
@@ -2631,28 +2643,28 @@
         <v>54</v>
       </c>
       <c r="B47" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C47" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="D47" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="E47" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="F47" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="G47" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="H47" t="s">
-        <v>277</v>
+        <v>280</v>
       </c>
       <c r="I47">
-        <v>28.8</v>
+        <v>27.5</v>
       </c>
     </row>
     <row r="48" spans="1:9">
@@ -2660,28 +2672,28 @@
         <v>55</v>
       </c>
       <c r="B48" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="C48" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="D48" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="E48" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="F48" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="G48" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="H48" t="s">
-        <v>278</v>
+        <v>281</v>
       </c>
       <c r="I48">
-        <v>16.8</v>
+        <v>28.8</v>
       </c>
     </row>
     <row r="49" spans="1:9">
@@ -2689,28 +2701,28 @@
         <v>56</v>
       </c>
       <c r="B49" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C49" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="D49" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="E49" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="F49" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="G49" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="H49" t="s">
-        <v>279</v>
+        <v>282</v>
       </c>
       <c r="I49">
-        <v>24.4</v>
+        <v>16.8</v>
       </c>
     </row>
     <row r="50" spans="1:9">
@@ -2718,28 +2730,28 @@
         <v>57</v>
       </c>
       <c r="B50" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C50" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="D50" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="E50" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="F50" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="G50" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="H50" t="s">
-        <v>280</v>
+        <v>283</v>
       </c>
       <c r="I50">
-        <v>14.2</v>
+        <v>24.4</v>
       </c>
     </row>
     <row r="51" spans="1:9">
@@ -2747,28 +2759,28 @@
         <v>58</v>
       </c>
       <c r="B51" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C51" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="D51" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="E51" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="F51" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="G51" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="H51" t="s">
-        <v>281</v>
+        <v>284</v>
       </c>
       <c r="I51">
-        <v>18.1</v>
+        <v>14.2</v>
       </c>
     </row>
     <row r="52" spans="1:9">
@@ -2776,28 +2788,28 @@
         <v>59</v>
       </c>
       <c r="B52" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C52" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="D52" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="E52" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="F52" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="G52" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="H52" t="s">
-        <v>282</v>
+        <v>285</v>
       </c>
       <c r="I52">
-        <v>15.9</v>
+        <v>18.1</v>
       </c>
     </row>
     <row r="53" spans="1:9">
@@ -2805,28 +2817,28 @@
         <v>60</v>
       </c>
       <c r="B53" t="s">
-        <v>120</v>
+        <v>135</v>
       </c>
       <c r="C53" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="D53" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="E53" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="F53" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="G53" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="H53" t="s">
-        <v>283</v>
+        <v>286</v>
       </c>
       <c r="I53">
-        <v>16.7</v>
+        <v>15.9</v>
       </c>
     </row>
     <row r="54" spans="1:9">
@@ -2834,28 +2846,28 @@
         <v>61</v>
       </c>
       <c r="B54" t="s">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="C54" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="D54" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="E54" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="F54" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="G54" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="H54" t="s">
-        <v>284</v>
+        <v>287</v>
       </c>
       <c r="I54">
-        <v>10.5</v>
+        <v>16.7</v>
       </c>
     </row>
     <row r="55" spans="1:9">
@@ -2863,28 +2875,28 @@
         <v>62</v>
       </c>
       <c r="B55" t="s">
-        <v>134</v>
+        <v>119</v>
       </c>
       <c r="C55" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="D55" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="E55" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="F55" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="G55" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="H55" t="s">
-        <v>285</v>
+        <v>288</v>
       </c>
       <c r="I55">
-        <v>20.8</v>
+        <v>10.5</v>
       </c>
     </row>
     <row r="56" spans="1:9">
@@ -2892,28 +2904,28 @@
         <v>63</v>
       </c>
       <c r="B56" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C56" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="D56" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="E56" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="F56" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="G56" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="H56" t="s">
-        <v>286</v>
+        <v>289</v>
       </c>
       <c r="I56">
-        <v>23.7</v>
+        <v>20.8</v>
       </c>
     </row>
     <row r="57" spans="1:9">
@@ -2921,28 +2933,28 @@
         <v>64</v>
       </c>
       <c r="B57" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C57" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="D57" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="E57" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="F57" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="G57" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="H57" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="I57">
-        <v>18.6</v>
+        <v>23.7</v>
       </c>
     </row>
     <row r="58" spans="1:9">
@@ -2950,28 +2962,28 @@
         <v>65</v>
       </c>
       <c r="B58" t="s">
-        <v>118</v>
+        <v>138</v>
       </c>
       <c r="C58" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="D58" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="E58" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="F58" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="G58" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="H58" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="I58">
-        <v>10.3</v>
+        <v>18.6</v>
       </c>
     </row>
     <row r="59" spans="1:9">
@@ -2979,28 +2991,28 @@
         <v>66</v>
       </c>
       <c r="B59" t="s">
-        <v>137</v>
+        <v>120</v>
       </c>
       <c r="C59" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="D59" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="E59" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="F59" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="G59" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="H59" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="I59">
-        <v>10.7</v>
+        <v>10.3</v>
       </c>
     </row>
     <row r="60" spans="1:9">
@@ -3008,28 +3020,28 @@
         <v>67</v>
       </c>
       <c r="B60" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C60" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="D60" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="E60" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="F60" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="G60" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="H60" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
       <c r="I60">
-        <v>5.7</v>
+        <v>10.7</v>
       </c>
     </row>
     <row r="61" spans="1:9">
@@ -3037,28 +3049,28 @@
         <v>68</v>
       </c>
       <c r="B61" t="s">
-        <v>121</v>
+        <v>140</v>
       </c>
       <c r="C61" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="D61" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="E61" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="F61" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="G61" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="H61" t="s">
-        <v>291</v>
+        <v>294</v>
       </c>
       <c r="I61">
-        <v>12.6</v>
+        <v>5.7</v>
       </c>
     </row>
     <row r="62" spans="1:9">
@@ -3066,28 +3078,28 @@
         <v>69</v>
       </c>
       <c r="B62" t="s">
-        <v>139</v>
+        <v>123</v>
       </c>
       <c r="C62" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="D62" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="E62" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="F62" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="G62" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="H62" t="s">
-        <v>292</v>
+        <v>295</v>
       </c>
       <c r="I62">
-        <v>21.8</v>
+        <v>12.6</v>
       </c>
     </row>
     <row r="63" spans="1:9">
@@ -3095,28 +3107,28 @@
         <v>70</v>
       </c>
       <c r="B63" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C63" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="D63" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="E63" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="F63" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="G63" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="H63" t="s">
-        <v>293</v>
+        <v>296</v>
       </c>
       <c r="I63">
-        <v>15.6</v>
+        <v>21.8</v>
       </c>
     </row>
     <row r="64" spans="1:9">
@@ -3124,28 +3136,28 @@
         <v>71</v>
       </c>
       <c r="B64" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="C64" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="D64" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="E64" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="F64" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="G64" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="H64" t="s">
-        <v>294</v>
+        <v>297</v>
       </c>
       <c r="I64">
-        <v>15.4</v>
+        <v>15.6</v>
       </c>
     </row>
     <row r="65" spans="1:9">
@@ -3153,28 +3165,28 @@
         <v>72</v>
       </c>
       <c r="B65" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C65" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="D65" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="E65" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="F65" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="G65" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="H65" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="I65">
-        <v>19.1</v>
+        <v>15.4</v>
       </c>
     </row>
     <row r="66" spans="1:9">
@@ -3182,28 +3194,28 @@
         <v>73</v>
       </c>
       <c r="B66" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="C66" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="D66" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="E66" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="F66" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="G66" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="H66" t="s">
-        <v>296</v>
+        <v>299</v>
       </c>
       <c r="I66">
-        <v>15.6</v>
+        <v>19.1</v>
       </c>
     </row>
     <row r="67" spans="1:9">
@@ -3211,28 +3223,28 @@
         <v>74</v>
       </c>
       <c r="B67" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C67" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="D67" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="E67" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="F67" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="G67" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="H67" t="s">
-        <v>297</v>
+        <v>300</v>
       </c>
       <c r="I67">
-        <v>13.7</v>
+        <v>15.6</v>
       </c>
     </row>
     <row r="68" spans="1:9">
@@ -3240,28 +3252,28 @@
         <v>75</v>
       </c>
       <c r="B68" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C68" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="D68" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="E68" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="F68" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="G68" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="H68" t="s">
-        <v>298</v>
+        <v>301</v>
       </c>
       <c r="I68">
-        <v>21.6</v>
+        <v>13.7</v>
       </c>
     </row>
     <row r="69" spans="1:9">
@@ -3269,28 +3281,28 @@
         <v>76</v>
       </c>
       <c r="B69" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="C69" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="D69" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="E69" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="F69" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="G69" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="H69" t="s">
-        <v>299</v>
+        <v>302</v>
       </c>
       <c r="I69">
-        <v>17</v>
+        <v>21.6</v>
       </c>
     </row>
     <row r="70" spans="1:9">
@@ -3298,28 +3310,28 @@
         <v>77</v>
       </c>
       <c r="B70" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C70" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="D70" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="E70" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="F70" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="G70" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="H70" t="s">
-        <v>300</v>
+        <v>303</v>
       </c>
       <c r="I70">
-        <v>20.6</v>
+        <v>17</v>
       </c>
     </row>
     <row r="71" spans="1:9">
@@ -3327,28 +3339,28 @@
         <v>78</v>
       </c>
       <c r="B71" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C71" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="D71" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="E71" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="F71" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="G71" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="H71" t="s">
-        <v>301</v>
+        <v>304</v>
       </c>
       <c r="I71">
-        <v>14.5</v>
+        <v>20.6</v>
       </c>
     </row>
     <row r="72" spans="1:9">
@@ -3356,28 +3368,28 @@
         <v>79</v>
       </c>
       <c r="B72" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="C72" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="D72" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="E72" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="F72" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="G72" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="H72" t="s">
-        <v>302</v>
+        <v>305</v>
       </c>
       <c r="I72">
-        <v>20.3</v>
+        <v>14.5</v>
       </c>
     </row>
     <row r="73" spans="1:9">
@@ -3385,28 +3397,28 @@
         <v>80</v>
       </c>
       <c r="B73" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="C73" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="D73" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="E73" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="F73" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="G73" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="H73" t="s">
-        <v>303</v>
+        <v>306</v>
       </c>
       <c r="I73">
-        <v>16.9</v>
+        <v>20.3</v>
       </c>
     </row>
     <row r="74" spans="1:9">
@@ -3414,28 +3426,28 @@
         <v>81</v>
       </c>
       <c r="B74" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C74" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="D74" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="E74" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="F74" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="G74" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="H74" t="s">
-        <v>304</v>
+        <v>307</v>
       </c>
       <c r="I74">
-        <v>11.2</v>
+        <v>16.9</v>
       </c>
     </row>
     <row r="75" spans="1:9">
@@ -3443,27 +3455,56 @@
         <v>82</v>
       </c>
       <c r="B75" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="C75" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="D75" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="E75" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="F75" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="G75" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="H75" t="s">
-        <v>305</v>
+        <v>308</v>
       </c>
       <c r="I75">
+        <v>11.2</v>
+      </c>
+    </row>
+    <row r="76" spans="1:9">
+      <c r="A76" t="s">
+        <v>83</v>
+      </c>
+      <c r="B76" t="s">
+        <v>154</v>
+      </c>
+      <c r="C76" t="s">
+        <v>157</v>
+      </c>
+      <c r="D76" t="s">
+        <v>162</v>
+      </c>
+      <c r="E76" t="s">
+        <v>165</v>
+      </c>
+      <c r="F76" t="s">
+        <v>229</v>
+      </c>
+      <c r="G76" t="s">
+        <v>236</v>
+      </c>
+      <c r="H76" t="s">
+        <v>309</v>
+      </c>
+      <c r="I76">
         <v>19.1</v>
       </c>
     </row>

</xml_diff>